<commit_message>
Replace fifth-Saturday availability with last_saturday.
Detect the last Saturday from the actual calendar date, update availability
cleaning/reporting labels, and refresh generated demo planning artifacts.
</commit_message>
<xml_diff>
--- a/data/raw/worship_availability_demo_en.xlsx
+++ b/data/raw/worship_availability_demo_en.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A622DB73-F685-49B7-8F24-6E41E2C66350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{16FD9CE1-0D47-46D1-B47A-65CDF34568C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="93">
   <si>
     <t>Timestamp</t>
   </si>
@@ -118,6 +118,9 @@
   </si>
   <si>
     <t>Saturday morning, Saturday afternoon</t>
+  </si>
+  <si>
+    <t>Last Saturday</t>
   </si>
   <si>
     <t>valentina.fuentes@example.com</t>
@@ -1058,7 +1061,9 @@
       <c r="I4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="4"/>
+      <c r="J4" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="K4" s="11"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1">
@@ -1066,10 +1071,10 @@
         <v>45821.789704594907</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D5" s="23"/>
       <c r="E5" s="5" t="s">
@@ -1082,16 +1087,16 @@
         <v>15</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1">
@@ -1099,32 +1104,32 @@
         <v>45821.94365465278</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" s="23"/>
       <c r="E6" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>15</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>17</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1">
@@ -1132,16 +1137,16 @@
         <v>45821.964541435183</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>14</v>
@@ -1156,7 +1161,7 @@
         <v>17</v>
       </c>
       <c r="J7" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K7" s="11"/>
     </row>
@@ -1165,10 +1170,10 @@
         <v>45821.970419884259</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D8" s="23"/>
       <c r="E8" s="3" t="s">
@@ -1181,16 +1186,16 @@
         <v>15</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>17</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1">
@@ -1198,31 +1203,31 @@
         <v>45822.83897527778</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J9" s="16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K9" s="11"/>
     </row>
@@ -1231,14 +1236,14 @@
         <v>45824.888788969911</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D10" s="23"/>
       <c r="E10" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>26</v>
@@ -1247,16 +1252,16 @@
         <v>15</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="J10" s="16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1">
@@ -1264,10 +1269,10 @@
         <v>45825.313125312503</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D11" s="23"/>
       <c r="E11" s="3" t="s">
@@ -1280,13 +1285,13 @@
         <v>15</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>22</v>
       </c>
       <c r="J11" s="17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K11" s="11"/>
     </row>
@@ -1295,30 +1300,30 @@
         <v>45826.802948888893</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>27</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>17</v>
       </c>
       <c r="J12" s="18"/>
       <c r="K12" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1">
@@ -1326,17 +1331,17 @@
         <v>45829.556947476849</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D13" s="23"/>
       <c r="E13" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>15</v>
@@ -1348,10 +1353,10 @@
         <v>17</v>
       </c>
       <c r="J13" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1">
@@ -1359,17 +1364,17 @@
         <v>45830.556947453704</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D14" s="23"/>
       <c r="E14" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>15</v>
@@ -1380,7 +1385,9 @@
       <c r="I14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J14" s="11"/>
+      <c r="J14" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1">
@@ -1388,29 +1395,29 @@
         <v>45831.556947453704</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D15" s="23"/>
       <c r="E15" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="J15" s="17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K15" s="10"/>
     </row>
@@ -1419,25 +1426,25 @@
         <v>45832.556947453704</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I16" s="14" t="s">
         <v>17</v>
@@ -1450,29 +1457,29 @@
         <v>45833.556947453704</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D17" s="23"/>
       <c r="E17" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G17" s="15" t="s">
         <v>27</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J17" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K17" s="10"/>
     </row>
@@ -1481,23 +1488,23 @@
         <v>45834.556947453704</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D18" s="23"/>
       <c r="E18" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
feat: add progressive planning relaxation and date ranges
- add configurable relaxation policies for frequency, directors, and roles
- support inclusive end dates and default warmup to zero
- make representative presence an explicit constraint
- improve band selection and generation reporting
- update pipeline documentation
</commit_message>
<xml_diff>
--- a/data/raw/worship_availability_demo_en.xlsx
+++ b/data/raw/worship_availability_demo_en.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16FD9CE1-0D47-46D1-B47A-65CDF34568C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4D389B7-BB04-4714-8FC5-788753970B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="94">
   <si>
     <t>Timestamp</t>
   </si>
@@ -45,6 +45,9 @@
     <t>Representative</t>
   </si>
   <si>
+    <t>Requires representative present</t>
+  </si>
+  <si>
     <t>Instrument</t>
   </si>
   <si>
@@ -168,7 +171,7 @@
     <t>Camila Miranda</t>
   </si>
   <si>
-    <t>Luke Miranda</t>
+    <t>Lucy Bennett</t>
   </si>
   <si>
     <t>Guitar, Vocals, Bass</t>
@@ -198,7 +201,7 @@
     <t>Gabriel Romero</t>
   </si>
   <si>
-    <t>Lucy Bennett</t>
+    <t>Lucas Romero</t>
   </si>
   <si>
     <t>Keyboard, Vocals</t>
@@ -623,7 +626,7 @@
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <font>
         <strike val="0"/>
@@ -653,6 +656,9 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -689,9 +695,9 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Respuestas de formulario 1-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="firstRowStripe" dxfId="4"/>
-      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -706,12 +712,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:K18" headerRowDxfId="2">
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:L18" headerRowDxfId="3">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Timestamp"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email" dataCellStyle="Hyperlink"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="First and Last Name"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Representative" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Representative" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{F92BF482-2053-4344-8CE1-A065589D2A1B}" name="Requires representative present" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Instrument"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Primary instrument" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name=" Director (Lead Vocals)"/>
@@ -925,22 +932,22 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K998"/>
+  <dimension ref="A1:L998"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
     <col min="3" max="3" width="18.85546875" customWidth="1"/>
-    <col min="4" max="4" width="31.5703125" customWidth="1"/>
-    <col min="5" max="6" width="31.42578125" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" customWidth="1"/>
-    <col min="8" max="8" width="101.5703125" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" customWidth="1"/>
-    <col min="10" max="10" width="111.7109375" customWidth="1"/>
-    <col min="11" max="11" width="127.140625" customWidth="1"/>
+    <col min="4" max="5" width="31.5703125" customWidth="1"/>
+    <col min="6" max="7" width="31.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" customWidth="1"/>
+    <col min="9" max="9" width="101.5703125" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" customWidth="1"/>
+    <col min="11" max="11" width="111.7109375" customWidth="1"/>
+    <col min="12" max="12" width="127.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="9" customFormat="1" ht="15.75" customHeight="1">
+    <row r="1" spans="1:12" s="9" customFormat="1" ht="15.75" customHeight="1">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -971,24 +978,25 @@
       <c r="J1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="19" t="s">
+      <c r="K1" s="8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1">
+      <c r="L1" s="19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="15.75" customHeight="1">
       <c r="A2" s="1">
         <v>45821.618713101852</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="23"/>
-      <c r="E2" s="5" t="s">
-        <v>13</v>
-      </c>
+      <c r="E2" s="23"/>
       <c r="F2" s="5" t="s">
         <v>14</v>
       </c>
@@ -1001,600 +1009,641 @@
       <c r="I2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="10"/>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1">
+      <c r="J2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="16"/>
+      <c r="L2" s="10"/>
+    </row>
+    <row r="3" spans="1:12" ht="15.75" customHeight="1">
       <c r="A3" s="2">
         <v>45821.62885479167</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" s="23"/>
-      <c r="E3" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="E3" s="23"/>
       <c r="F3" s="3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="17" t="s">
+      <c r="J3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="11"/>
-    </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1">
+      <c r="K3" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="11"/>
+    </row>
+    <row r="4" spans="1:12" ht="15.75" customHeight="1">
       <c r="A4" s="2">
         <v>45821.726428842587</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D4" s="23"/>
-      <c r="E4" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="E4" s="23"/>
       <c r="F4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="4" t="s">
+      <c r="I4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="11"/>
-    </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1">
+      <c r="J4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L4" s="11"/>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" customHeight="1">
       <c r="A5" s="1">
         <v>45821.789704594907</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" s="23"/>
-      <c r="E5" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="E5" s="23"/>
       <c r="F5" s="5" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="K5" s="16" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1">
+      <c r="L5" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" customHeight="1">
       <c r="A6" s="2">
         <v>45821.94365465278</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="23"/>
-      <c r="E6" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="E6" s="23"/>
       <c r="F6" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="J6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" s="17" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1">
+      <c r="L6" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" customHeight="1">
       <c r="A7" s="1">
         <v>45821.964541435183</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="D7" t="s">
         <v>46</v>
       </c>
+      <c r="E7" s="24" t="s">
+        <v>16</v>
+      </c>
       <c r="F7" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="K7" s="11"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1">
+      <c r="J7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="11"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" customHeight="1">
       <c r="A8" s="2">
         <v>45821.970419884259</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" s="23"/>
-      <c r="E8" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="E8" s="23"/>
       <c r="F8" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="J8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" s="17" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1">
+      <c r="L8" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" customHeight="1">
       <c r="A9" s="1">
         <v>45822.83897527778</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="D9" s="24" t="s">
         <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>28</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>57</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J9" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="K9" s="11"/>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1">
+      <c r="J9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9" s="11"/>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" customHeight="1">
       <c r="A10" s="1">
         <v>45824.888788969911</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D10" s="23"/>
-      <c r="E10" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="E10" s="23"/>
       <c r="F10" s="5" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K10" s="10" t="s">
+      <c r="J10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="16" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1">
+      <c r="L10" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" customHeight="1">
       <c r="A11" s="2">
         <v>45825.313125312503</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="D11" s="23"/>
-      <c r="E11" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="E11" s="23"/>
       <c r="F11" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J11" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="K11" s="11"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1">
+        <v>59</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="L11" s="11"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.75" customHeight="1">
       <c r="A12" s="13">
         <v>45826.802948888893</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D12" s="23"/>
-      <c r="E12" s="14" t="s">
-        <v>70</v>
-      </c>
+      <c r="E12" s="23"/>
       <c r="F12" s="14" t="s">
         <v>71</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="I12" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" s="18"/>
-      <c r="K12" s="10" t="s">
+      <c r="H12" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1">
+      <c r="J12" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" s="18"/>
+      <c r="L12" s="10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15.75" customHeight="1">
       <c r="A13" s="12">
         <v>45829.556947476849</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D13" s="23"/>
-      <c r="E13" s="10" t="s">
-        <v>76</v>
-      </c>
+      <c r="E13" s="23"/>
       <c r="F13" s="10" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="K13" s="10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1">
+        <v>29</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="15.75" customHeight="1">
       <c r="A14" s="12">
         <v>45830.556947453704</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D14" s="23"/>
-      <c r="E14" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>39</v>
+      <c r="E14" s="23"/>
+      <c r="F14" s="5" t="s">
+        <v>47</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J14" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="K14" s="10"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1">
+      <c r="J14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="L14" s="10"/>
+    </row>
+    <row r="15" spans="1:12" ht="15.75" customHeight="1">
       <c r="A15" s="12">
         <v>45831.556947453704</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D15" s="23"/>
-      <c r="E15" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>57</v>
+      <c r="E15" s="23"/>
+      <c r="F15" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>50</v>
+        <v>58</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>16</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J15" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="K15" s="10"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1">
+        <v>51</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="L15" s="10"/>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" customHeight="1">
       <c r="A16" s="12">
         <v>45832.556947453704</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F16" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>57</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I16" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="11"/>
-      <c r="K16" s="10"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.75" customHeight="1">
+      <c r="H16" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="K16" s="11"/>
+      <c r="L16" s="10"/>
+    </row>
+    <row r="17" spans="1:12" ht="15.75" customHeight="1">
       <c r="A17" s="12">
         <v>45833.556947453704</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D17" s="23"/>
-      <c r="E17" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="G17" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="H17" s="3" t="s">
+      <c r="E17" s="23"/>
+      <c r="F17" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="I17" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J17" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K17" s="10"/>
-    </row>
-    <row r="18" spans="1:11" ht="15.75" customHeight="1">
+      <c r="H17" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K17" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="L17" s="10"/>
+    </row>
+    <row r="18" spans="1:12" ht="15.75" customHeight="1">
       <c r="A18" s="12">
         <v>45834.556947453704</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D18" s="23"/>
-      <c r="E18" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>71</v>
+      <c r="E18" s="23"/>
+      <c r="F18" s="3" t="s">
+        <v>93</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J18" s="11"/>
-      <c r="K18" s="10"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="22" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1">
+        <v>72</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K18" s="11"/>
+      <c r="L18" s="10"/>
+    </row>
+    <row r="19" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="20" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="21" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="22" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="23" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="25" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="26" spans="1:12" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:12" ht="15.75" customHeight="1">
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
       <c r="D27" s="22"/>
-    </row>
-    <row r="28" spans="1:11" ht="15.75" customHeight="1">
+      <c r="E27" s="22"/>
+    </row>
+    <row r="28" spans="1:12" ht="15.75" customHeight="1">
       <c r="B28" s="21"/>
       <c r="D28" s="23"/>
-    </row>
-    <row r="29" spans="1:11" ht="15.75" customHeight="1">
+      <c r="E28" s="23"/>
+    </row>
+    <row r="29" spans="1:12" ht="15.75" customHeight="1">
       <c r="B29" s="21"/>
       <c r="D29" s="23"/>
-    </row>
-    <row r="30" spans="1:11" ht="15.75" customHeight="1">
+      <c r="E29" s="23"/>
+    </row>
+    <row r="30" spans="1:12" ht="15.75" customHeight="1">
       <c r="B30" s="21"/>
       <c r="D30" s="23"/>
-    </row>
-    <row r="31" spans="1:11" ht="15.75" customHeight="1">
+      <c r="E30" s="23"/>
+    </row>
+    <row r="31" spans="1:12" ht="15.75" customHeight="1">
       <c r="B31" s="21"/>
       <c r="D31" s="23"/>
-    </row>
-    <row r="32" spans="1:11" ht="15.75" customHeight="1">
+      <c r="E31" s="23"/>
+    </row>
+    <row r="32" spans="1:12" ht="15.75" customHeight="1">
       <c r="B32" s="21"/>
       <c r="D32" s="23"/>
-    </row>
-    <row r="33" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E32" s="23"/>
+    </row>
+    <row r="33" spans="2:5" ht="15.75" customHeight="1">
       <c r="B33" s="21"/>
       <c r="D33" s="24"/>
-    </row>
-    <row r="34" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E33" s="24"/>
+    </row>
+    <row r="34" spans="2:5" ht="15.75" customHeight="1">
       <c r="B34" s="21"/>
       <c r="D34" s="23"/>
-    </row>
-    <row r="35" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E34" s="23"/>
+    </row>
+    <row r="35" spans="2:5" ht="15.75" customHeight="1">
       <c r="B35" s="21"/>
     </row>
-    <row r="36" spans="2:4" ht="15.75" customHeight="1">
+    <row r="36" spans="2:5" ht="15.75" customHeight="1">
       <c r="B36" s="21"/>
       <c r="D36" s="23"/>
-    </row>
-    <row r="37" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E36" s="23"/>
+    </row>
+    <row r="37" spans="2:5" ht="15.75" customHeight="1">
       <c r="B37" s="21"/>
       <c r="D37" s="23"/>
-    </row>
-    <row r="38" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E37" s="23"/>
+    </row>
+    <row r="38" spans="2:5" ht="15.75" customHeight="1">
       <c r="B38" s="21"/>
       <c r="D38" s="23"/>
-    </row>
-    <row r="39" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E38" s="23"/>
+    </row>
+    <row r="39" spans="2:5" ht="15.75" customHeight="1">
       <c r="B39" s="21"/>
       <c r="D39" s="23"/>
-    </row>
-    <row r="40" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E39" s="23"/>
+    </row>
+    <row r="40" spans="2:5" ht="15.75" customHeight="1">
       <c r="B40" s="21"/>
       <c r="D40" s="23"/>
-    </row>
-    <row r="41" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E40" s="23"/>
+    </row>
+    <row r="41" spans="2:5" ht="15.75" customHeight="1">
       <c r="B41" s="21"/>
       <c r="D41" s="23"/>
-    </row>
-    <row r="42" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E41" s="23"/>
+    </row>
+    <row r="42" spans="2:5" ht="15.75" customHeight="1">
       <c r="B42" s="21"/>
     </row>
-    <row r="43" spans="2:4" ht="15.75" customHeight="1">
+    <row r="43" spans="2:5" ht="15.75" customHeight="1">
       <c r="B43" s="21"/>
       <c r="D43" s="23"/>
-    </row>
-    <row r="44" spans="2:4" ht="15.75" customHeight="1">
+      <c r="E43" s="23"/>
+    </row>
+    <row r="44" spans="2:5" ht="15.75" customHeight="1">
       <c r="B44" s="21"/>
       <c r="D44" s="23"/>
-    </row>
-    <row r="45" spans="2:4" ht="15.75" customHeight="1"/>
-    <row r="46" spans="2:4" ht="15.75" customHeight="1"/>
-    <row r="47" spans="2:4" ht="15.75" customHeight="1"/>
-    <row r="48" spans="2:4" ht="15.75" customHeight="1"/>
+      <c r="E44" s="23"/>
+    </row>
+    <row r="45" spans="2:5" ht="15.75" customHeight="1"/>
+    <row r="46" spans="2:5" ht="15.75" customHeight="1"/>
+    <row r="47" spans="2:5" ht="15.75" customHeight="1"/>
+    <row r="48" spans="2:5" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
@@ -2553,7 +2602,7 @@
     <hyperlink ref="B5" r:id="rId4" xr:uid="{DAB9AFB7-EA52-4EE4-8ABF-0C7C8CD35CDA}"/>
     <hyperlink ref="B6" r:id="rId5" xr:uid="{0EC236D1-F281-41CE-A6F5-625545656E09}"/>
     <hyperlink ref="B7" r:id="rId6" xr:uid="{96BA4D58-1A96-4520-831F-872E44203BAA}"/>
-    <hyperlink ref="D7" r:id="rId7" display="luke.miranda@example.com" xr:uid="{C450BA37-526C-4D6A-B41E-F60F63F8852F}"/>
+    <hyperlink ref="D9" r:id="rId7" display="luke.miranda@example.com" xr:uid="{C450BA37-526C-4D6A-B41E-F60F63F8852F}"/>
     <hyperlink ref="B8" r:id="rId8" xr:uid="{6C26E5F0-7E07-4D0B-BC44-734B8E79D0F1}"/>
     <hyperlink ref="B9" r:id="rId9" xr:uid="{92C63CBA-9819-41DE-A1EA-7C4B375495D3}"/>
     <hyperlink ref="B10" r:id="rId10" xr:uid="{8CAD868C-30B9-4C0A-86A5-26D0B2E0E6F1}"/>

</xml_diff>